<commit_message>
docs: corregir inconsistencias del modelo de datos del mvp
</commit_message>
<xml_diff>
--- a/Docs/Dev/Moica - Diccionario de Datos.xlsx
+++ b/Docs/Dev/Moica - Diccionario de Datos.xlsx
@@ -8178,7 +8178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -8265,9 +8265,8 @@
           <t>Restricciones BD</t>
         </is>
       </c>
-      <c r="E5" s="8">
-        <f>COUNTA(B24:B24)</f>
-        <v/>
+      <c r="E5" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="G5" s="84" t="inlineStr">
         <is>
@@ -8536,7 +8535,7 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Aplicación</t>
+          <t>Base de datos</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
@@ -8880,6 +8879,51 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="38" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>ckCambioEstadoSolicitudTransicion</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>estadoAnterior, estadoNuevo</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>estadoNuevo &lt;&gt; estadoAnterior; el registro inicial admite estadoAnterior nulo.</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="E4:F4"/>
@@ -9748,7 +9792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -9835,9 +9879,8 @@
           <t>Restricciones BD</t>
         </is>
       </c>
-      <c r="E5" s="8">
-        <f>COUNTA(B26:B29)</f>
-        <v/>
+      <c r="E5" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="G5" s="84" t="inlineStr">
         <is>
@@ -10106,7 +10149,7 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Aplicación</t>
+          <t>Base de datos</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
@@ -10567,27 +10610,27 @@
       </c>
     </row>
     <row r="28" ht="38" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>UQ</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>uqCalificacionUsuarioSolicitudCalificado</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>idSolicitudServicio, idCalificado</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Cada participante recibe como máximo una calificación por solicitud.</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>Base de datos</t>
         </is>
@@ -10601,25 +10644,67 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
+          <t>ckCalificacionUsuarioParticipantes</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>idCalificador, idCalificado</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>idCalificador &lt;&gt; idCalificado.</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="38" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
           <t>ckCalificacionUsuarioPuntuacion</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>puntuacion</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>puntuacion BETWEEN 1 AND 5.</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>Base de datos</t>
         </is>
       </c>
     </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="E4:F4"/>

</xml_diff>

<commit_message>
docs: alinear los nombres de entidades con el diccionario de datos
</commit_message>
<xml_diff>
--- a/Docs/Dev/Moica - Diccionario de Datos.xlsx
+++ b/Docs/Dev/Moica - Diccionario de Datos.xlsx
@@ -8178,7 +8178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -8265,8 +8265,9 @@
           <t>Restricciones BD</t>
         </is>
       </c>
-      <c r="E5" s="8" t="n">
-        <v>2</v>
+      <c r="E5" s="8">
+        <f>COUNTA(B24:B25)</f>
+        <v/>
       </c>
       <c r="G5" s="84" t="inlineStr">
         <is>
@@ -8906,24 +8907,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="E4:F4"/>
@@ -9792,7 +9775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -9879,8 +9862,9 @@
           <t>Restricciones BD</t>
         </is>
       </c>
-      <c r="E5" s="8" t="n">
-        <v>5</v>
+      <c r="E5" s="8">
+        <f>COUNTA(B26:B30)</f>
+        <v/>
       </c>
       <c r="G5" s="84" t="inlineStr">
         <is>
@@ -10690,21 +10674,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="E4:F4"/>

</xml_diff>

<commit_message>
docs(db): ajustar reglas de verificacion al formato del diccionario
</commit_message>
<xml_diff>
--- a/Docs/Dev/Moica - Diccionario de Datos.xlsx
+++ b/Docs/Dev/Moica - Diccionario de Datos.xlsx
@@ -2505,7 +2505,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="38" customHeight="1">
+    <row r="32" ht="46" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
           <t>PK</t>
@@ -2532,7 +2532,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="38" customHeight="1">
+    <row r="33" ht="46" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>CK</t>
@@ -5439,7 +5439,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="38" customHeight="1">
+    <row r="28" ht="46" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>PK</t>
@@ -5466,7 +5466,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="38" customHeight="1">
+    <row r="29" ht="46" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>UQ</t>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Índice único parcial WHERE estadoSolicitud IN ('PENDIENTE', 'EN_REVISION'): una sola solicitud abierta por nivel y perfil.</t>
+          <t>Índice parcial: una solicitud abierta por perfil y nivel.</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -5493,7 +5493,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="38" customHeight="1">
+    <row r="30" ht="46" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
         <is>
           <t>CK</t>
@@ -5520,7 +5520,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="38" customHeight="1">
+    <row r="31" ht="46" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t>CK</t>
@@ -5547,7 +5547,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="38" customHeight="1">
+    <row r="32" ht="46" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
         <is>
           <t>CK</t>
@@ -5565,7 +5565,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Los estados RECHAZADA y REVOCADA exigen una observación no vacía.</t>
+          <t>RECHAZADA y REVOCADA exigen una observación no vacía.</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -5574,7 +5574,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="38" customHeight="1">
+    <row r="33" ht="46" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>CK</t>
@@ -5592,7 +5592,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>fechaInicioRevision y fechaResolucion no pueden ser anteriores a fechaSolicitud, y los estados finales exigen fechaResolucion.</t>
+          <t>Revisión y resolución nunca preceden a fechaSolicitud.</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
@@ -5606,8 +5606,8 @@
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A26:J26"/>
     <mergeCell ref="A20:J20"/>
-    <mergeCell ref="A26:J26"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="G5:J5"/>
     <mergeCell ref="B4:C4"/>
@@ -6312,7 +6312,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="38" customHeight="1">
+    <row r="24" ht="46" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>PK</t>
@@ -6339,7 +6339,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="38" customHeight="1">
+    <row r="25" ht="46" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>UQ</t>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>La clave de almacenamiento identifica un único archivo privado.</t>
+          <t>La clave de almacenamiento identifica un único archivo.</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -6366,7 +6366,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="38" customHeight="1">
+    <row r="26" ht="46" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>CK</t>
@@ -6393,7 +6393,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="38" customHeight="1">
+    <row r="27" ht="46" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>CK</t>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>tipoMime IN ('image/jpeg', 'image/png', 'application/pdf').</t>
+          <t>Solo image/jpeg, image/png y application/pdf.</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -6420,7 +6420,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="38" customHeight="1">
+    <row r="28" ht="46" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
           <t>CK</t>

</xml_diff>